<commit_message>
Added Assignments 1 and 2
</commit_message>
<xml_diff>
--- a/Components and Finance List.xlsx
+++ b/Components and Finance List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aseblr-my.sharepoint.com/personal/bl_en_u4rae23003_bl_students_amrita_edu/Documents/College/Duck/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="116" documentId="8_{059E5F43-FE72-450E-8E5C-434BF849694A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50B61C74-5240-4983-B4E2-9BF4F9A34678}"/>
+  <xr:revisionPtr revIDLastSave="117" documentId="8_{059E5F43-FE72-450E-8E5C-434BF849694A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4DD6457-3B72-479A-83BF-865BE46E338F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E7439860-74A8-42DE-9746-8BE225D34625}"/>
   </bookViews>
@@ -214,20 +214,20 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -599,7 +599,7 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="5" t="s">
         <v>35</v>
       </c>
     </row>
@@ -685,7 +685,7 @@
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="6">
         <v>46063</v>
       </c>
       <c r="C5" t="s">
@@ -718,7 +718,7 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="6"/>
+      <c r="B6" s="7"/>
       <c r="C6" t="s">
         <v>21</v>
       </c>
@@ -797,7 +797,7 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="7"/>
+      <c r="B9" s="9"/>
       <c r="C9" t="s">
         <v>33</v>
       </c>
@@ -823,7 +823,7 @@
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="7"/>
+      <c r="B10" s="9"/>
       <c r="C10" t="s">
         <v>34</v>
       </c>
@@ -842,7 +842,7 @@
       </c>
       <c r="L10">
         <f>(L9-F15)</f>
-        <v>7827.25</v>
+        <v>7827</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
@@ -856,11 +856,11 @@
         <v>1</v>
       </c>
       <c r="E11">
-        <v>643.75</v>
+        <v>644</v>
       </c>
       <c r="F11">
         <f t="shared" si="0"/>
-        <v>643.75</v>
+        <v>644</v>
       </c>
       <c r="H11" t="s">
         <v>37</v>
@@ -884,7 +884,7 @@
       </c>
       <c r="F15">
         <f>SUM(F1:F13)</f>
-        <v>14172.75</v>
+        <v>14173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added simple CV code
</commit_message>
<xml_diff>
--- a/Components and Finance List.xlsx
+++ b/Components and Finance List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aseblr-my.sharepoint.com/personal/bl_en_u4rae23003_bl_students_amrita_edu/Documents/College/Duck/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="117" documentId="8_{059E5F43-FE72-450E-8E5C-434BF849694A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4DD6457-3B72-479A-83BF-865BE46E338F}"/>
+  <xr:revisionPtr revIDLastSave="127" documentId="8_{059E5F43-FE72-450E-8E5C-434BF849694A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1D426BE-6345-4997-B65F-DFADEDB44483}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E7439860-74A8-42DE-9746-8BE225D34625}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>Sl. No.</t>
   </si>
@@ -150,6 +150,15 @@
   </si>
   <si>
     <t>White</t>
+  </si>
+  <si>
+    <t>Screws and Inserts</t>
+  </si>
+  <si>
+    <t>Screws, Inserts and Magnets</t>
+  </si>
+  <si>
+    <t>OnlyScrews</t>
   </si>
 </sst>
 </file>
@@ -564,7 +573,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04AFD439-7064-4EC4-9939-FB45E41C4017}">
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="15.109375" style="2" customWidth="1"/>
@@ -644,7 +653,7 @@
         <v>206</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F13" si="0">D3*E3</f>
+        <f t="shared" ref="F3:F14" si="0">D3*E3</f>
         <v>206</v>
       </c>
       <c r="G3" t="s">
@@ -841,8 +850,8 @@
         <v>27</v>
       </c>
       <c r="L10">
-        <f>(L9-F15)</f>
-        <v>7827</v>
+        <f>(L9-F16)</f>
+        <v>7555</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
@@ -867,9 +876,30 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3">
+        <v>46104</v>
+      </c>
+      <c r="C12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>272</v>
+      </c>
       <c r="F12">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>272</v>
+      </c>
+      <c r="G12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H12" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
@@ -878,13 +908,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="E15" t="s">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="F14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E16" t="s">
         <v>28</v>
       </c>
-      <c r="F15">
-        <f>SUM(F1:F13)</f>
-        <v>14173</v>
+      <c r="F16">
+        <f>SUM(F1:F14)</f>
+        <v>14445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added 2 more assignments
</commit_message>
<xml_diff>
--- a/Components and Finance List.xlsx
+++ b/Components and Finance List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aseblr-my.sharepoint.com/personal/bl_en_u4rae23003_bl_students_amrita_edu/Documents/College/Duck/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="127" documentId="8_{059E5F43-FE72-450E-8E5C-434BF849694A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1D426BE-6345-4997-B65F-DFADEDB44483}"/>
+  <xr:revisionPtr revIDLastSave="134" documentId="8_{059E5F43-FE72-450E-8E5C-434BF849694A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03475A8E-D165-4DBA-94F4-14B12F19D994}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E7439860-74A8-42DE-9746-8BE225D34625}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Sl. No.</t>
   </si>
@@ -159,6 +159,9 @@
   </si>
   <si>
     <t>OnlyScrews</t>
+  </si>
+  <si>
+    <t>Dynamixel Motors</t>
   </si>
 </sst>
 </file>
@@ -720,7 +723,7 @@
         <v>20</v>
       </c>
       <c r="L5">
-        <v>22000</v>
+        <v>28624</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -825,7 +828,7 @@
       </c>
       <c r="L9">
         <f>SUM(L5:L7)</f>
-        <v>22000</v>
+        <v>28624</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
@@ -851,7 +854,7 @@
       </c>
       <c r="L10">
         <f>(L9-F16)</f>
-        <v>7555</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
@@ -903,9 +906,24 @@
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3">
+        <v>46122</v>
+      </c>
+      <c r="C13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13">
+        <v>4</v>
+      </c>
+      <c r="E13">
+        <v>2906</v>
+      </c>
       <c r="F13">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>11624</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
@@ -920,7 +938,7 @@
       </c>
       <c r="F16">
         <f>SUM(F1:F14)</f>
-        <v>14445</v>
+        <v>26069</v>
       </c>
     </row>
   </sheetData>

</xml_diff>